<commit_message>
add electrical cable, worm shalft
</commit_message>
<xml_diff>
--- a/Measurements/HL3M10 3-projection hex weld nuts/HL3M10.xlsx
+++ b/Measurements/HL3M10 3-projection hex weld nuts/HL3M10.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\manoe\Meng\solidworks\Measurements\HL3M10 3-projection hex weld nuts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF2073BA-F5FB-4615-BA6F-38CE0B3C2286}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6AC77DD-6968-4F12-8572-207BB095ED79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{32BFC42B-CD3D-49FE-8254-52B3F518DB85}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="38">
   <si>
     <t>Customer</t>
   </si>
@@ -1336,11 +1336,21 @@
       <c r="H8" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="I8" s="2"/>
-      <c r="J8" s="2"/>
-      <c r="K8" s="2"/>
-      <c r="L8" s="2"/>
-      <c r="M8" s="2"/>
+      <c r="I8" s="2">
+        <v>0.99</v>
+      </c>
+      <c r="J8" s="2">
+        <v>1.08</v>
+      </c>
+      <c r="K8" s="2">
+        <v>1.05</v>
+      </c>
+      <c r="L8" s="2">
+        <v>1.07</v>
+      </c>
+      <c r="M8" s="2">
+        <v>1.05</v>
+      </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
@@ -1366,14 +1376,24 @@
         <f t="shared" si="1"/>
         <v>1.67</v>
       </c>
-      <c r="H9" s="3"/>
+      <c r="H9" s="3" t="s">
+        <v>37</v>
+      </c>
       <c r="I9" s="2">
         <v>1.74</v>
       </c>
-      <c r="J9" s="2"/>
-      <c r="K9" s="2"/>
-      <c r="L9" s="2"/>
-      <c r="M9" s="2"/>
+      <c r="J9" s="2">
+        <v>1.75</v>
+      </c>
+      <c r="K9" s="2">
+        <v>1.8</v>
+      </c>
+      <c r="L9" s="2">
+        <v>1.78</v>
+      </c>
+      <c r="M9" s="2">
+        <v>1.83</v>
+      </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
@@ -1399,18 +1419,30 @@
         <f t="shared" si="1"/>
         <v>13.299999999999999</v>
       </c>
-      <c r="H10" s="3"/>
-      <c r="I10" s="2"/>
-      <c r="J10" s="2"/>
-      <c r="K10" s="2"/>
-      <c r="L10" s="2"/>
-      <c r="M10" s="2"/>
+      <c r="H10" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="I10" s="2">
+        <v>13.45</v>
+      </c>
+      <c r="J10" s="2">
+        <v>13.44</v>
+      </c>
+      <c r="K10" s="2">
+        <v>13.42</v>
+      </c>
+      <c r="L10" s="2">
+        <v>13.41</v>
+      </c>
+      <c r="M10" s="2">
+        <v>13.41</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="G1:G3"/>
   </mergeCells>
-  <conditionalFormatting sqref="I5:M10">
+  <conditionalFormatting sqref="I5:M6 I8:M10">
     <cfRule type="cellIs" dxfId="1" priority="22" operator="notBetween">
       <formula>$G5</formula>
       <formula>$F5</formula>

</xml_diff>